<commit_message>
CORE-000093: address review comments
Add negative test coverage for --DOSU absent from the dataset entirely
(not just null) by removing the ECDOSU column from ec.xpt and
validating/highlighting the resulting errors. Also reorder
Description/Message to state the condition before the violation,
per reviewer feedback.
</commit_message>
<xml_diff>
--- a/rules/CORE-000093/negative/01/data/unit-test-coreid-CG0114-negative.xlsx
+++ b/rules/CORE-000093/negative/01/data/unit-test-coreid-CG0114-negative.xlsx
@@ -1111,7 +1111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1527,6 +1527,11 @@
           <t>ECDOSU</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>[ABSENT]</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2034,6 +2039,272 @@
       <c r="E36" t="inlineStr">
         <is>
           <t>SUDOSU</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>8</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>5</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>ECTRT</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>BOTTLE A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>8</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>5</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>ECDOSE</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>8</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>5</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>ECDOSTXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>8</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>5</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>ECDOSTOT</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>[ABSENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>8</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>5</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>ECDOSU</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>[ABSENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>9</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>8</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>ECTRT</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>BOTTLE A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>9</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>8</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>ECDOSE</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>9</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>8</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>ECDOSTXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>9</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>8</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>ECDOSTOT</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>[ABSENT]</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>9</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>ec.xpt</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>8</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>ECDOSU</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>[ABSENT]</t>
         </is>
       </c>
     </row>
@@ -2964,7 +3235,6 @@
       <c r="K11" s="7" t="str"/>
       <c r="L11" s="7" t="str"/>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="I13" s="7" t="str"/>
       <c r="J13" s="7" t="str"/>
@@ -2985,7 +3255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:P8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3046,30 +3316,25 @@
       </c>
       <c r="L1" s="5" t="inlineStr">
         <is>
-          <t>ECDOSU</t>
+          <t>ECDOSFRM</t>
         </is>
       </c>
       <c r="M1" s="5" t="inlineStr">
         <is>
-          <t>ECDOSFRM</t>
+          <t>ECSTDTC</t>
         </is>
       </c>
       <c r="N1" s="5" t="inlineStr">
         <is>
-          <t>ECSTDTC</t>
+          <t>ECENDTC</t>
         </is>
       </c>
       <c r="O1" s="5" t="inlineStr">
         <is>
-          <t>ECENDTC</t>
+          <t>ECSTDY</t>
         </is>
       </c>
       <c r="P1" s="5" t="inlineStr">
-        <is>
-          <t>ECSTDY</t>
-        </is>
-      </c>
-      <c r="Q1" s="5" t="inlineStr">
         <is>
           <t>ECENDY</t>
         </is>
@@ -3133,30 +3398,25 @@
       </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>Dose Units</t>
+          <t>Dose Form</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr">
         <is>
-          <t>Dose Form</t>
+          <t>Start Date/Time of Treatment</t>
         </is>
       </c>
       <c r="N2" s="8" t="inlineStr">
         <is>
-          <t>Start Date/Time of Treatment</t>
+          <t>End Date/Time of Treatment</t>
         </is>
       </c>
       <c r="O2" s="8" t="inlineStr">
         <is>
-          <t>End Date/Time of Treatment</t>
+          <t>Study Day of Start of Treatment</t>
         </is>
       </c>
       <c r="P2" s="8" t="inlineStr">
-        <is>
-          <t>Study Day of Start of Treatment</t>
-        </is>
-      </c>
-      <c r="Q2" s="8" t="inlineStr">
         <is>
           <t>Study Day of End of Treatment</t>
         </is>
@@ -3235,15 +3495,10 @@
       </c>
       <c r="O3" s="8" t="inlineStr">
         <is>
-          <t>Char</t>
+          <t>Num</t>
         </is>
       </c>
       <c r="P3" s="8" t="inlineStr">
-        <is>
-          <t>Num</t>
-        </is>
-      </c>
-      <c r="Q3" s="8" t="inlineStr">
         <is>
           <t>Num</t>
         </is>
@@ -3293,14 +3548,11 @@
         <v>50</v>
       </c>
       <c r="O4" s="8" t="n">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="P4" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="Q4" s="8" t="n">
-        <v>8</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3326,7 +3578,7 @@
           <t>A2-20110114</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="11" t="inlineStr">
         <is>
           <t>BOTTLE A</t>
         </is>
@@ -3341,34 +3593,29 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J5" t="n">
+      <c r="J5" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="K5" s="7" t="str"/>
+      <c r="K5" s="12" t="str"/>
       <c r="L5" t="inlineStr">
         <is>
-          <t>TABLET</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
           <t>QD</t>
         </is>
       </c>
+      <c r="M5" s="7" t="inlineStr">
+        <is>
+          <t>2011-01-14</t>
+        </is>
+      </c>
       <c r="N5" s="7" t="inlineStr">
         <is>
-          <t>2011-01-14</t>
-        </is>
-      </c>
-      <c r="O5" s="7" t="inlineStr">
-        <is>
           <t>2011-01-28</t>
         </is>
       </c>
+      <c r="O5" t="n">
+        <v>1</v>
+      </c>
       <c r="P5" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q5" t="n">
         <v>15</v>
       </c>
     </row>
@@ -3415,26 +3662,25 @@
         <v>2</v>
       </c>
       <c r="K6" s="12" t="str"/>
-      <c r="L6" s="11" t="str"/>
-      <c r="M6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>QD</t>
         </is>
       </c>
+      <c r="M6" s="7" t="inlineStr">
+        <is>
+          <t>2011-01-14</t>
+        </is>
+      </c>
       <c r="N6" s="7" t="inlineStr">
         <is>
-          <t>2011-01-14</t>
-        </is>
-      </c>
-      <c r="O6" s="7" t="inlineStr">
-        <is>
           <t>2011-01-23</t>
         </is>
       </c>
+      <c r="O6" t="n">
+        <v>1</v>
+      </c>
       <c r="P6" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q6" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3485,30 +3731,25 @@
       <c r="K7" s="7" t="str"/>
       <c r="L7" t="inlineStr">
         <is>
-          <t>TABLET</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
           <t>QD</t>
         </is>
       </c>
+      <c r="M7" s="7" t="inlineStr">
+        <is>
+          <t>2011-01-24</t>
+        </is>
+      </c>
       <c r="N7" s="7" t="inlineStr">
         <is>
           <t>2011-01-24</t>
         </is>
       </c>
-      <c r="O7" s="7" t="inlineStr">
-        <is>
-          <t>2011-01-24</t>
-        </is>
+      <c r="O7" t="n">
+        <v>11</v>
       </c>
       <c r="P7" t="n">
         <v>11</v>
       </c>
-      <c r="Q7" t="n">
-        <v>11</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3534,7 +3775,7 @@
           <t>A2-20110125</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="11" t="inlineStr">
         <is>
           <t>BOTTLE A</t>
         </is>
@@ -3549,34 +3790,29 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="J8" t="n">
+      <c r="J8" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="K8" s="7" t="str"/>
+      <c r="K8" s="12" t="str"/>
       <c r="L8" t="inlineStr">
         <is>
-          <t>TABLET</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
           <t>QD</t>
         </is>
       </c>
+      <c r="M8" s="7" t="inlineStr">
+        <is>
+          <t>2011-01-25</t>
+        </is>
+      </c>
       <c r="N8" s="7" t="inlineStr">
         <is>
-          <t>2011-01-25</t>
-        </is>
-      </c>
-      <c r="O8" s="7" t="inlineStr">
-        <is>
           <t>2011-01-28</t>
         </is>
       </c>
+      <c r="O8" t="n">
+        <v>12</v>
+      </c>
       <c r="P8" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q8" t="n">
         <v>15</v>
       </c>
     </row>

</xml_diff>